<commit_message>
Mise à jour et simplification des Agents 6 et 7 avec intégration LLM Gemini
</commit_message>
<xml_diff>
--- a/AGENT6/outputs/cost_analysis.xlsx
+++ b/AGENT6/outputs/cost_analysis.xlsx
@@ -419,7 +419,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Poste de dépense</t>
+          <t>Poste</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
@@ -435,7 +435,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>765000</v>
+        <v>714000</v>
       </c>
     </row>
     <row r="3">

</xml_diff>